<commit_message>
resolve: accept remote cache files from pipeline run
</commit_message>
<xml_diff>
--- a/Job_Hunt_Tracker.xlsx
+++ b/Job_Hunt_Tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -128,6 +128,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -495,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y10"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -653,22 +659,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>2026-06-23 22:29</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Ripjar</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>Product Manager</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>Remote (Global)</t>
         </is>
@@ -678,80 +684,80 @@
           <t>Ripjar was founded by veterans of GCHQ to bring national security-grade intelligence tools to the fight against financial crime. Financial crime funds human trafficking, terrorism, corruption and sanctions evasion on a global scale, and the organisations on the front line need technology built to match the threat.&lt;br&gt;&lt;br&gt;Today, Ripjar's AI-native software and data fusion products are used by governments, the world's largest banks, and global enterprises to automate the detection, investigation and monitoring of serious financial crime. Every day, hundreds of customers and thousands of daily active users rely on the platform to screen hundreds of millions of names for risk...</t>
         </is>
       </c>
-      <c r="F2" s="17" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-product-manager-ripjar-1133665</t>
         </is>
       </c>
-      <c r="G2" s="16" t="n">
+      <c r="G2" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="H2" s="16" t="n">
+      <c r="H2" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="I2" s="16" t="n">
+      <c r="I2" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J2" s="16" t="inlineStr">
+      <c r="J2" s="20" t="inlineStr">
         <is>
           <t>GOOD FIT</t>
         </is>
       </c>
-      <c r="K2" s="16" t="inlineStr">
+      <c r="K2" s="20" t="inlineStr">
         <is>
           <t>Hiring Team</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
+      <c r="L2" s="20" t="inlineStr">
         <is>
           <t>Recruitment</t>
         </is>
       </c>
-      <c r="M2" s="16" t="inlineStr">
+      <c r="M2" s="20" t="inlineStr">
         <is>
           <t>recruitment@ripjar.com</t>
         </is>
       </c>
-      <c r="N2" s="16" t="inlineStr">
+      <c r="N2" s="20" t="inlineStr">
         <is>
           <t>hr_alias</t>
         </is>
       </c>
-      <c r="O2" s="16" t="inlineStr">
+      <c r="O2" s="20" t="inlineStr">
         <is>
           <t>sent</t>
         </is>
       </c>
-      <c r="P2" s="16" t="inlineStr">
+      <c r="P2" s="20" t="inlineStr">
         <is>
           <t>Aman_Sharma_Resume_Ripjar.pdf</t>
         </is>
       </c>
-      <c r="Q2" s="16" t="inlineStr"/>
-      <c r="R2" s="16" t="inlineStr"/>
-      <c r="S2" s="17" t="inlineStr">
+      <c r="Q2" s="20" t="inlineStr"/>
+      <c r="R2" s="20" t="inlineStr"/>
+      <c r="S2" s="21" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-product-manager-ripjar-1133665</t>
         </is>
       </c>
-      <c r="T2" s="16" t="inlineStr">
+      <c r="T2" s="20" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="U2" s="16" t="inlineStr"/>
-      <c r="V2" s="16" t="inlineStr"/>
-      <c r="W2" s="16" t="inlineStr">
+      <c r="U2" s="20" t="inlineStr"/>
+      <c r="V2" s="20" t="inlineStr"/>
+      <c r="W2" s="20" t="inlineStr">
         <is>
           <t>Touch 1</t>
         </is>
       </c>
-      <c r="X2" s="16" t="inlineStr">
+      <c r="X2" s="20" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="Y2" s="16" t="inlineStr">
+      <c r="Y2" s="20" t="inlineStr">
         <is>
           <t>Find real contact</t>
         </is>
@@ -760,66 +766,62 @@
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>2026-06-25 06:34</t>
+          <t>2026-06-25 13:59</t>
         </is>
       </c>
       <c r="B3" s="18" t="inlineStr">
         <is>
-          <t>Toyota Connected Europe</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Data Product Owner</t>
-        </is>
-      </c>
-      <c r="D3" s="18" t="inlineStr">
-        <is>
-          <t>London, England, United Kingdom</t>
-        </is>
-      </c>
+          <t>Business Analyst - Data &amp; AI</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Permanent Farringdon, London - Hybrid Are you a dynamic and experience Technical Product Owner interesting in leading one of our product team in the realm of connected mobility? Essential experience for this role includes working with data pipelines and data points. What is the role? The Technical Product Owner is engaged short-term to perform a structured gap analysis for a technical project and translate findings into clear, testable requirements that engineering teams can estimate, plan, and deliver. The role ensure the target state is well-defined and the path to get there is unambiguous. What will you do? - Requirements Pack:...</t>
+          <t>Why Valtech? We’re the experience innovation company - a trusted partner to the world’s most recognized brands. To our people we offer growth opportunities, a values-driven culture, international careers and the chance to shape the future of experience.The opportunityAt Valtech, you’ll find an environment designed for continuous learning, meaningful impact, and professional growth. Whether you're pioneering new digital solutions, challenging conventional thinking or building the next generation of customer experiences, your work will help transform industries.We Are Proud OfThe work we do and the innovation we drive Our values of share, care and dare A workplace culture that fosters creativity,...</t>
         </is>
       </c>
       <c r="F3" s="19" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/data-product-owner-at-toyota-connected-europe-4431830840?position=33&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=mv1XfXn48FHlQxlaWEPobw%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4421818265</t>
         </is>
       </c>
       <c r="G3" s="18" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="H3" s="18" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I3" s="18" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="J3" s="18" t="inlineStr">
         <is>
-          <t>PARTIAL FIT</t>
+          <t>STRONG FIT</t>
         </is>
       </c>
       <c r="K3" s="18" t="inlineStr">
         <is>
-          <t>Hiring Team</t>
+          <t>Sheree Atcheson</t>
         </is>
       </c>
       <c r="L3" s="18" t="inlineStr">
         <is>
-          <t>Recruitment</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="M3" s="18" t="inlineStr">
         <is>
-          <t>recruitment@toyotaconnectedeurope.com</t>
+          <t>sheree.atcheson@valtech.com</t>
         </is>
       </c>
       <c r="N3" s="18" t="inlineStr">
         <is>
-          <t>hr_alias</t>
+          <t>website_scrape</t>
         </is>
       </c>
       <c r="O3" s="18" t="inlineStr">
@@ -829,14 +831,14 @@
       </c>
       <c r="P3" s="18" t="inlineStr">
         <is>
-          <t>Aman_Sharma_Resume_Toyota_Connected_Europe.pdf</t>
+          <t>Aman_Sharma_Resume_Valtech.pdf</t>
         </is>
       </c>
       <c r="Q3" s="18" t="inlineStr"/>
       <c r="R3" s="18" t="inlineStr"/>
       <c r="S3" s="19" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/data-product-owner-at-toyota-connected-europe-4431830840?position=33&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=mv1XfXn48FHlQxlaWEPobw%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4421818265</t>
         </is>
       </c>
       <c r="T3" s="18" t="inlineStr">
@@ -858,178 +860,170 @@
       </c>
       <c r="Y3" s="18" t="inlineStr">
         <is>
-          <t>Find real contact</t>
+          <t>Follow-up Day 5</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>2026-06-25 06:34</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Mediatech</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>Vilnius, Vilniaus, Lithuania</t>
-        </is>
-      </c>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:00</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Capco</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>AI Business Analyst - Glasgow/Edinburgh</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>MEDIATECH Mediatech is one of the fastest-growing digital publishing houses, reaching over 25 million people every month across Cybernews, Wellness Pulse, InvestorsObserver, and our wider network. We deliver trusted, independently researched insights across tech, cybersecurity, health, and finance. Our investigations have exposed major security issues at NASA, WhatsApp, ChatGPT, PayPal, LinkedIn, and the Red Cross, and uncovered the largest-ever password leak (RockYou2024). We’re a team driven by curiosity, impact, and fast growth - and we’re looking for people who want to build with us. PRODUCT TEAM Our Product Management team works closely with the Development team to turn business ideas...</t>
-        </is>
-      </c>
-      <c r="F4" s="17" t="inlineStr">
-        <is>
-          <t>https://lt.linkedin.com/jobs/view/product-owner-at-mediatech-4432542351?position=38&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=94rvlKUzhquz0Fj9xVsVdw%3D%3D</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="H4" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="I4" s="16" t="n">
+          <t>AI Business Analyst –Location Glasgow (Hybrid) | Type: PermanentDrive impactful change within Scotland’s Financial sectorThe RoleCapco is seeking experienced Business Analysts to join our Business Consulting practice, supporting strategic transformation programmes across leading financial services and investment banking clients. This role combines core business analysis expertise with a focus on AI-enabled transformation, helping clients bridge the gap between emerging AI capabilities and practical business outcomes.Working closely with business stakeholders, product teams, AI specialists, and technology delivery teams, you will identify opportunities to leverage Generative AI, automation, and agentic workflows to improve operational efficiency, employee productivity, decision-making, and customer outcomes. You...</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4421801929</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>61</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="I4" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>GOOD FIT</t>
         </is>
       </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>Hiring Team</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>Recruitment</t>
-        </is>
-      </c>
-      <c r="M4" s="16" t="inlineStr">
-        <is>
-          <t>recruitment@mediatech.com</t>
-        </is>
-      </c>
-      <c r="N4" s="16" t="inlineStr">
-        <is>
-          <t>hr_alias</t>
-        </is>
-      </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>Tim Steele</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="M4" s="20" t="inlineStr">
+        <is>
+          <t>tim.steele@capco.com</t>
+        </is>
+      </c>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
+          <t>website_scrape</t>
+        </is>
+      </c>
+      <c r="O4" s="20" t="inlineStr">
         <is>
           <t>sent</t>
         </is>
       </c>
-      <c r="P4" s="16" t="inlineStr">
-        <is>
-          <t>Aman_Sharma_Resume_Mediatech.pdf</t>
-        </is>
-      </c>
-      <c r="Q4" s="16" t="inlineStr"/>
-      <c r="R4" s="16" t="inlineStr"/>
-      <c r="S4" s="17" t="inlineStr">
-        <is>
-          <t>https://lt.linkedin.com/jobs/view/product-owner-at-mediatech-4432542351?position=38&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=94rvlKUzhquz0Fj9xVsVdw%3D%3D</t>
-        </is>
-      </c>
-      <c r="T4" s="16" t="inlineStr">
+      <c r="P4" s="20" t="inlineStr">
+        <is>
+          <t>Aman_Sharma_Resume_Capco.pdf</t>
+        </is>
+      </c>
+      <c r="Q4" s="20" t="inlineStr"/>
+      <c r="R4" s="20" t="inlineStr"/>
+      <c r="S4" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4421801929</t>
+        </is>
+      </c>
+      <c r="T4" s="20" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="U4" s="16" t="inlineStr"/>
-      <c r="V4" s="16" t="inlineStr"/>
-      <c r="W4" s="16" t="inlineStr">
+      <c r="U4" s="20" t="inlineStr"/>
+      <c r="V4" s="20" t="inlineStr"/>
+      <c r="W4" s="20" t="inlineStr">
         <is>
           <t>Touch 1</t>
         </is>
       </c>
-      <c r="X4" s="16" t="inlineStr">
+      <c r="X4" s="20" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="Y4" s="16" t="inlineStr">
-        <is>
-          <t>Find real contact</t>
+      <c r="Y4" s="20" t="inlineStr">
+        <is>
+          <t>Follow-up Day 5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>2026-06-25 06:34</t>
+          <t>2026-06-25 14:00</t>
         </is>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Clario</t>
+          <t>DataBeat.io Media</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Budapest, Hungary</t>
-        </is>
-      </c>
+          <t>Senior Data Analyst</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>At Clario, part of Thermo Fisher Scientific, we develop regulated technology that helps unlock better evidence and improve patient outcomes worldwide. Our software platforms support clinical trials, diagnostics, and medical decision‑making in highly controlled regulatory environments. As a Product Owner, you will play a critical role in driving product delivery and ensuring that Agile teams effectively translate product vision into high-quality, executable work. You will collaborate closely with Product Management, Engineering, and cross-functional stakeholders to manage the team backlog, refine requirements, and deliver value aligned with business needs and customer expectations. What We Offer - Competitive compensation - SZÉP Card...</t>
+          <t>Job Title: Senior Data Analyst – AdTech (Team Lead)Location: HyderabadExperience Level: 4–6 YearsEmployment Type: Full-timeShift Timings: 5PM - 2AM ISTAbout The RoleWe are looking for a highly experienced and hands-on Senior Data Analyst (AdTech) to lead our analytics team. This role is ideal for someone with a strong background in log-level data handling, cross-platform data engineering, and a solid command of modern BI tools. You'll play a key role in building scalable data pipelines, leading analytics strategy, and mentoring a team of analysts.Key ResponsibilitiesLead and mentor a team of data analysts, ensuring quality delivery and technical upskilling.Design, develop, and maintain...</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>https://hu.linkedin.com/jobs/view/product-owner-at-clario-4432544759?position=44&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=0qCmrMulcNmaqUpI%2F9J3kA%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4405491561</t>
         </is>
       </c>
       <c r="G5" s="18" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="J5" s="18" t="inlineStr">
         <is>
-          <t>GOOD FIT</t>
+          <t>PARTIAL FIT</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
         <is>
-          <t>Tünde Sztojov</t>
+          <t>Hiring Team</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>Talent Acquisition Partner at Clario | Clinical Trials and Technology Opportunities</t>
+          <t>Recruitment</t>
         </is>
       </c>
       <c r="M5" s="18" t="inlineStr">
         <is>
-          <t>tnde.sztojov@clarioinc.com</t>
+          <t>recruitment@databeatiomedia.com</t>
         </is>
       </c>
       <c r="N5" s="18" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>hr_alias</t>
         </is>
       </c>
       <c r="O5" s="18" t="inlineStr">
@@ -1039,14 +1033,14 @@
       </c>
       <c r="P5" s="18" t="inlineStr">
         <is>
-          <t>Aman_Sharma_Resume_Clario.pdf</t>
+          <t>Aman_Sharma_Resume_DataBeat_io_Media.pdf</t>
         </is>
       </c>
       <c r="Q5" s="18" t="inlineStr"/>
       <c r="R5" s="18" t="inlineStr"/>
       <c r="S5" s="19" t="inlineStr">
         <is>
-          <t>https://hu.linkedin.com/jobs/view/product-owner-at-clario-4432544759?position=44&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=0qCmrMulcNmaqUpI%2F9J3kA%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4405491561</t>
         </is>
       </c>
       <c r="T5" s="18" t="inlineStr">
@@ -1068,110 +1062,106 @@
       </c>
       <c r="Y5" s="18" t="inlineStr">
         <is>
-          <t>Follow-up Day 5</t>
+          <t>Find real contact</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>2026-06-25 06:35</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Lenstra</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Paris, Île-de-France, France</t>
-        </is>
-      </c>
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:00</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Mphasis</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Principal Business Analyst</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Lenstra was created by the passion of engineers specialised in Computer Science with a proven history in delivering top quality solutions to its customers. Bringing together work excellence and vision we managed to serve top tier clients from a variety of industry domains like Banking/Insurance, Luxury and Tech. We help our clients to solve their most difficult problems around Cloud Computing &amp;amp; DevOps, Data Platform, IT Security by having a holistic approach of their environment and building often complex but always relevant solutions to help them accelerate their business. Our engineering team is committed to great ethics and most of...</t>
-        </is>
-      </c>
-      <c r="F6" s="17" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/technical-product-owner-at-lenstra-4429864041?position=15&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=wGLXANVkv5e5OdGoRANTtQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="I6" s="16" t="n">
+          <t>Senior Business Analyst / Product Owner Experience: 8–12 YearsRole SummaryLead business analysis and product ownership for AI/ML‑driven enterprise initiatives. Drive requirement strategy, stakeholder alignment, product roadmap detailing, and support full AI/ML lifecycle delivery.Key ResponsibilitiesLead and own requirement strategy: BRD, FRD, SRS, Epics, Features, User Stories.Conduct advanced current/future‑state modeling, gap analysis, and business impact assessment.Drive backlog prioritization, roadmap planning, and executive‑level stakeholder alignment.Partner with AI/ML teams on problem framing, feature engineering, model evaluation, and business validation.Lead workshops, UAT sessions, demos, and executive briefings.Oversee governance documentation: traceability matrices, business rules, data dictionaries, process flows.Support end‑to‑end AI/ML lifecycle: Business Understanding → Data →...</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4414277494</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>61</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="I6" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J6" s="16" t="inlineStr">
+      <c r="J6" s="20" t="inlineStr">
         <is>
           <t>GOOD FIT</t>
         </is>
       </c>
-      <c r="K6" s="16" t="inlineStr">
+      <c r="K6" s="20" t="inlineStr">
         <is>
           <t>Hiring Team</t>
         </is>
       </c>
-      <c r="L6" s="16" t="inlineStr">
+      <c r="L6" s="20" t="inlineStr">
         <is>
           <t>Recruitment</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr">
-        <is>
-          <t>recruitment@lenstra.com</t>
-        </is>
-      </c>
-      <c r="N6" s="16" t="inlineStr">
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>recruitment@mphasis.com</t>
+        </is>
+      </c>
+      <c r="N6" s="20" t="inlineStr">
         <is>
           <t>hr_alias</t>
         </is>
       </c>
-      <c r="O6" s="16" t="inlineStr">
+      <c r="O6" s="20" t="inlineStr">
         <is>
           <t>sent</t>
         </is>
       </c>
-      <c r="P6" s="16" t="inlineStr">
-        <is>
-          <t>Aman_Sharma_Resume_Lenstra.pdf</t>
-        </is>
-      </c>
-      <c r="Q6" s="16" t="inlineStr"/>
-      <c r="R6" s="16" t="inlineStr"/>
-      <c r="S6" s="17" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/technical-product-owner-at-lenstra-4429864041?position=15&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=wGLXANVkv5e5OdGoRANTtQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="T6" s="16" t="inlineStr">
+      <c r="P6" s="20" t="inlineStr">
+        <is>
+          <t>Aman_Sharma_Resume_Mphasis.pdf</t>
+        </is>
+      </c>
+      <c r="Q6" s="20" t="inlineStr"/>
+      <c r="R6" s="20" t="inlineStr"/>
+      <c r="S6" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4414277494</t>
+        </is>
+      </c>
+      <c r="T6" s="20" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="U6" s="16" t="inlineStr"/>
-      <c r="V6" s="16" t="inlineStr"/>
-      <c r="W6" s="16" t="inlineStr">
+      <c r="U6" s="20" t="inlineStr"/>
+      <c r="V6" s="20" t="inlineStr"/>
+      <c r="W6" s="20" t="inlineStr">
         <is>
           <t>Touch 1</t>
         </is>
       </c>
-      <c r="X6" s="16" t="inlineStr">
+      <c r="X6" s="20" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="Y6" s="16" t="inlineStr">
+      <c r="Y6" s="20" t="inlineStr">
         <is>
           <t>Find real contact</t>
         </is>
@@ -1180,39 +1170,35 @@
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>2026-06-25 06:36</t>
+          <t>2026-06-25 14:01</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>RJ-Search</t>
+          <t>DataBeat</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Product Owner - Onboarding</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Norwich, England, United Kingdom</t>
-        </is>
-      </c>
+          <t>Senior Data Analyst</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Product Owner - Onboarding &amp;amp; Platform Location: Norwich&amp;nbsp; Epos Now powers over 100,000 businesses globally through integrated POS, payments and commerce solutions. We're looking for a Product Owner to take ownership of one of the most important parts of the customer journey: onboarding. From account creation and identity verification through to system configuration and activation, you'll help shape how merchants get up and running and realise value from day one. This role sits at the intersection of product, engineering, design, payments and operations. You'll use customer insight, behavioural data and commercial thinking to identify friction points, prioritise improvements and deliver...</t>
+          <t>Job Title: Senior Data Analyst – AdTech (Team Lead)Location: HyderabadExperience Level: 4–6 YearsEmployment Type: Full-timeShift Timings: 5PM - 2AM ISTAbout The RoleWe are looking for a highly experienced and hands-on Senior Data Analyst (AdTech) to lead our analytics team. This role is ideal for someone with a strong background in log-level data handling, cross-platform data engineering, and a solid command of modern BI tools. You'll play a key role in building scalable data pipelines, leading analytics strategy, and mentoring a team of analysts.Key ResponsibilitiesLead and mentor a team of data analysts, ensuring quality delivery and technical upskilling.Design, develop, and maintain...</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/product-owner-onboarding-at-rj-search-4432579955?position=31&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=c0RBC0VK%2F6CCiZH4mLWP3A%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4249614593</t>
         </is>
       </c>
       <c r="G7" s="18" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H7" s="18" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="I7" s="18" t="n">
         <v>62</v>
@@ -1234,7 +1220,7 @@
       </c>
       <c r="M7" s="18" t="inlineStr">
         <is>
-          <t>recruitment@rjsearch.com</t>
+          <t>recruitment@databeat.com</t>
         </is>
       </c>
       <c r="N7" s="18" t="inlineStr">
@@ -1249,14 +1235,14 @@
       </c>
       <c r="P7" s="18" t="inlineStr">
         <is>
-          <t>Aman_Sharma_Resume_RJ-Search.pdf</t>
+          <t>Aman_Sharma_Resume_DataBeat.pdf</t>
         </is>
       </c>
       <c r="Q7" s="18" t="inlineStr"/>
       <c r="R7" s="18" t="inlineStr"/>
       <c r="S7" s="19" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/product-owner-onboarding-at-rj-search-4432579955?position=31&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=c0RBC0VK%2F6CCiZH4mLWP3A%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4249614593</t>
         </is>
       </c>
       <c r="T7" s="18" t="inlineStr">
@@ -1283,160 +1269,152 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>2026-06-25 06:36</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>BNP Paribas Fortis</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Brussels, Brussels Region, Belgium</t>
-        </is>
-      </c>
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Robert Walters</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Data Platform Squad Lead | Agile Delivery | Investment Banking</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>YOUR JOB IN A NUTSHELL As a Product Owner you play a pivotal role in shaping the future of your product and contribute to impactful initiatives that make a tangible difference in the lives of our customers and employees. As the bridge between stakeholders and IT, you’ll turn strategic vision into actionable solutions, driving value creation in an Agile environment. You will be part of the Transformation Office at BNP Paribas Fortis, which is the driving force behind the bank’s strategic evolution. With a clear mission to guide the bank’s transformation, we focus on value creation, operational simplicity, efficiency and...</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/jobs/view/product-owner-at-bnp-paribas-fortis-4408730495?position=48&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=dlmtSURYTh%2FunLFR%2B9JAJA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="I8" s="16" t="n">
-        <v>58</v>
-      </c>
-      <c r="J8" s="16" t="inlineStr">
+          <t>Robert Walters is delighted to be partnering with a leading international banking group on the appointment of a Data Platform Squad Lead to join their expanding Data &amp; Analytics Technology function in Dublin.This is a leadership opportunity for an experienced Data Platform Delivery Lead, Technical Product Owner or Agile Data Manager to drive the delivery of strategic data platform initiatives supporting Corporate and Investment Banking operations across EMEA.The OpportunityAs Data Platform Squad Lead, you will take ownership of a cross-functional data delivery squad comprising Architects, Business Analysts, Data Engineers, Developers, Testers, Data Modellers and Data Governance specialists.Acting as the bridge...</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4428498158</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>53</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>62</v>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
         <is>
           <t>PARTIAL FIT</t>
         </is>
       </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>Sarah Bekkaoui</t>
-        </is>
-      </c>
-      <c r="L8" s="16" t="inlineStr">
-        <is>
-          <t>Talent Acquisition Consultant | RPO | BNP Paribas Fortis</t>
-        </is>
-      </c>
-      <c r="M8" s="16" t="inlineStr">
-        <is>
-          <t>sarah.bekkaoui@bnpparibasfortis.com</t>
-        </is>
-      </c>
-      <c r="N8" s="16" t="inlineStr">
-        <is>
-          <t>pattern</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="inlineStr">
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>Hiring Team</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="M8" s="20" t="inlineStr">
+        <is>
+          <t>recruitment@robertwalters.com</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
+          <t>hr_alias</t>
+        </is>
+      </c>
+      <c r="O8" s="20" t="inlineStr">
         <is>
           <t>sent</t>
         </is>
       </c>
-      <c r="P8" s="16" t="inlineStr">
-        <is>
-          <t>Aman_Sharma_Resume_BNP_Paribas_Fortis.pdf</t>
-        </is>
-      </c>
-      <c r="Q8" s="16" t="inlineStr"/>
-      <c r="R8" s="16" t="inlineStr"/>
-      <c r="S8" s="17" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/jobs/view/product-owner-at-bnp-paribas-fortis-4408730495?position=48&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=dlmtSURYTh%2FunLFR%2B9JAJA%3D%3D</t>
-        </is>
-      </c>
-      <c r="T8" s="16" t="inlineStr">
+      <c r="P8" s="20" t="inlineStr">
+        <is>
+          <t>Aman_Sharma_Resume_Robert_Walters.pdf</t>
+        </is>
+      </c>
+      <c r="Q8" s="20" t="inlineStr"/>
+      <c r="R8" s="20" t="inlineStr"/>
+      <c r="S8" s="21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4428498158</t>
+        </is>
+      </c>
+      <c r="T8" s="20" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="U8" s="16" t="inlineStr"/>
-      <c r="V8" s="16" t="inlineStr"/>
-      <c r="W8" s="16" t="inlineStr">
+      <c r="U8" s="20" t="inlineStr"/>
+      <c r="V8" s="20" t="inlineStr"/>
+      <c r="W8" s="20" t="inlineStr">
         <is>
           <t>Touch 1</t>
         </is>
       </c>
-      <c r="X8" s="16" t="inlineStr">
+      <c r="X8" s="20" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="Y8" s="16" t="inlineStr">
-        <is>
-          <t>Follow-up Day 5</t>
+      <c r="Y8" s="20" t="inlineStr">
+        <is>
+          <t>Find real contact</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>2026-06-25 06:36</t>
+          <t>2026-06-25 14:02</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>C Teleport</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Product Owner - Back Office, Integration &amp; Ecosystem</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Rotterdam, South Holland, Netherlands</t>
-        </is>
-      </c>
+          <t>Senior Specialist, LCS Product Business Analyst</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Are you a Product Owner who has built integrations that genuinely eliminate manual work — not just connect systems, but remove the human effort between them? Do you understand how operational data flows across scheduling, HR, expense, and finance tools? Can you translate complex customer workflows into integration logic that works reliably at scale? If so, we'd love to meet you. At C Teleport, we manage high-volume, high-stakes crew travel for maritime, aviation, and energy operators. In this environment, manual work is not just inefficient — it is a risk. Our integration layer exists to eliminate it: automating data flows...</t>
+          <t>Job DescriptionThe OpportunityBased in Hyderabad, join a global healthcare biopharma company and be part of a 130- year legacy of success backed by ethical integrity, forward momentum, and an inspiring mission to achieve new milestones in global healthcare. Be part of an organisation driven by digital technology and data-backed approaches that support a diversified portfolio of prescription medicines, vaccines, and animal health products. Drive innovation and execution excellence. Be a part of a team with passion for using data, analytics, and insights to drive decision-making, and which creates custom software, allowing us to tackle some of the world's greatest health...</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/product-owner-back-office-integration-ecosystem-at-c-teleport-4432843420?position=55&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=oWJ8UsnsqojBAUe1cA4I%2BQ%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4431359239</t>
         </is>
       </c>
       <c r="G9" s="18" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="H9" s="18" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>LOW FIT</t>
+          <t>PARTIAL FIT</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr"/>
       <c r="L9" s="18" t="inlineStr"/>
       <c r="M9" s="18" t="inlineStr">
         <is>
-          <t>info@cteleport.com</t>
+          <t>mediarelations@msd.com</t>
         </is>
       </c>
       <c r="N9" s="18" t="inlineStr">
@@ -1451,14 +1429,14 @@
       </c>
       <c r="P9" s="18" t="inlineStr">
         <is>
-          <t>Aman_Sharma_Resume_C_Teleport.pdf</t>
+          <t>Aman_Sharma_Resume_MSD.pdf</t>
         </is>
       </c>
       <c r="Q9" s="18" t="inlineStr"/>
       <c r="R9" s="18" t="inlineStr"/>
       <c r="S9" s="19" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/product-owner-back-office-integration-ecosystem-at-c-teleport-4432843420?position=55&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=oWJ8UsnsqojBAUe1cA4I%2BQ%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4431359239</t>
         </is>
       </c>
       <c r="T9" s="18" t="inlineStr">
@@ -1487,58 +1465,62 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-06-25 06:36</t>
+          <t>2026-06-25 14:02</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>TP ICAP</t>
+          <t>Delta Technology Hub</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>London, England, United Kingdom</t>
-        </is>
-      </c>
+          <t>Senior Data Analyst</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>he TP ICAP Group is a world leading provider of market infrastructure. Our purpose is to provide clients with access to global financial and commodities markets, improving price discovery, liquidity, and distribution of data, through responsible and innovative solutions. Through our people and technology, we connect clients to superior liquidity and data solutions. The Group is home to a stable of premium brands. Collectively, TP ICAP is the largest interdealer broker in the world by revenue, the number one Energy &amp;amp; Commodities broker in the world, the world’s leading provider of OTC data, and an award winning all-to-all trading platform....</t>
+          <t>How You'll Help Us Keep Climbing (Overview &amp; Key Responsibilities)Role SummaryDelta Air Lines is seeking a talented and motivated Senior Data Analyst to join their HR innovation and employee experience team. This role is perfect for someone with a deep understanding of data modelling best practices, strong technical skills, and business acumen, as well as the ability to learn complex data models and apply that knowledge to solve real-world business challenges. You will work on the development of data models to integrate, aggregate, and harmonize HR data from various sources, while driving the migration to modern platforms like Python and...</t>
         </is>
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/product-owner-at-tp-icap-4410188065?position=20&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=UkYTHCgoHJ6goRNpYsoWQg%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4404207279</t>
         </is>
       </c>
       <c r="G10" s="20" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="J10" s="20" t="inlineStr">
         <is>
-          <t>LOW FIT</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr"/>
-      <c r="L10" s="20" t="inlineStr"/>
+          <t>PARTIAL FIT</t>
+        </is>
+      </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>Hiring Team</t>
+        </is>
+      </c>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
       <c r="M10" s="20" t="inlineStr">
         <is>
-          <t>askhrrecruitmentamers@tpicap.com</t>
+          <t>recruitment@deltahub.com</t>
         </is>
       </c>
       <c r="N10" s="20" t="inlineStr">
         <is>
-          <t>website_scrape</t>
+          <t>hr_alias</t>
         </is>
       </c>
       <c r="O10" s="20" t="inlineStr">
@@ -1548,14 +1530,14 @@
       </c>
       <c r="P10" s="20" t="inlineStr">
         <is>
-          <t>Aman_Sharma_Resume_TP_ICAP.pdf</t>
+          <t>Aman_Sharma_Resume_Delta_Technology_Hub.pdf</t>
         </is>
       </c>
       <c r="Q10" s="20" t="inlineStr"/>
       <c r="R10" s="20" t="inlineStr"/>
       <c r="S10" s="21" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/jobs/view/product-owner-at-tp-icap-4410188065?position=20&amp;pageNum=0&amp;refId=6%2B93z1YJ%2FPHoCdIcWzIc3w%3D%3D&amp;trackingId=UkYTHCgoHJ6goRNpYsoWQg%3D%3D</t>
+          <t>https://www.linkedin.com/jobs/view/4404207279</t>
         </is>
       </c>
       <c r="T10" s="20" t="inlineStr">
@@ -1576,6 +1558,103 @@
         </is>
       </c>
       <c r="Y10" s="20" t="inlineStr">
+        <is>
+          <t>Find real contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:02</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>London Area, United Kingdom</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Job Title: Business Analyst – London Market Insurance / Specialty InsuranceExp Required – 8 years Plus Location: LondonDomain London Market Insurance / Lloyd’s Market / Specialty Insurance / Commercial Insurance Location About the Job you are considering:We are looking for an experienced Business Analyst with strong London Market Insurance domain expertise to support business and technology transformation initiatives for a specialty insurance client. The candidate should have strong experience across London Market insurance processes, including underwriting, claims, policy administration, delegated authority, bordereaux, reinsurance, premium processing, regulatory reporting, data, and system transformation. The ideal candidate should be able to work closely...</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423125476</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>27</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="J11" s="22" t="inlineStr">
+        <is>
+          <t>LOW FIT</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="inlineStr"/>
+      <c r="L11" s="22" t="inlineStr"/>
+      <c r="M11" s="22" t="inlineStr">
+        <is>
+          <t>name@capgemini.com</t>
+        </is>
+      </c>
+      <c r="N11" s="22" t="inlineStr">
+        <is>
+          <t>website_scrape</t>
+        </is>
+      </c>
+      <c r="O11" s="22" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="P11" s="22" t="inlineStr">
+        <is>
+          <t>Aman_Sharma_Resume_Capgemini.pdf</t>
+        </is>
+      </c>
+      <c r="Q11" s="22" t="inlineStr"/>
+      <c r="R11" s="22" t="inlineStr"/>
+      <c r="S11" s="23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423125476</t>
+        </is>
+      </c>
+      <c r="T11" s="22" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="U11" s="22" t="inlineStr"/>
+      <c r="V11" s="22" t="inlineStr"/>
+      <c r="W11" s="22" t="inlineStr">
+        <is>
+          <t>Touch 1</t>
+        </is>
+      </c>
+      <c r="X11" s="22" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="Y11" s="22" t="inlineStr">
         <is>
           <t>Follow-up Day 5</t>
         </is>
@@ -1601,6 +1680,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>